<commit_message>
Update QA Testing Matrix to explicitly document siren volume hardware limitations for warning commands
</commit_message>
<xml_diff>
--- a/QA_TEST_MATRIX.xlsx
+++ b/QA_TEST_MATRIX.xlsx
@@ -638,12 +638,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>1-SECOND GENTLE CHIME on sirens.</t>
+          <t>1-SECOND CHIME on sirens.</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Simulates a simple door opening.</t>
+          <t>HARDWARE LIMITATION: Siren ignores low-volume setting and always plays loud.</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Warning chime for light impacts.</t>
+          <t>HARDWARE LIMITATION: Siren ignores low-volume setting and always plays loud.</t>
         </is>
       </c>
     </row>
@@ -912,7 +912,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Levels: 0=Low, 1=Medium, 2=High, 3=Very High.</t>
+          <t>Levels: 0=Low, 1=Medium, 2=High, 3=Very High. Note: Some firmwares ignore volume.</t>
         </is>
       </c>
     </row>
@@ -929,7 +929,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Provide mode 1-6 to test a specific sound (1=Burglar, 2=Fire, 3=Emergency, 4=Police Panic, 5=Fire Panic, 6=Emergency Panic).</t>
+          <t>Provide mode 1-6 to test a specific sound.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Configure Onics Button properly as IAS Zone Panic Button via Manufacturer Specific Write
</commit_message>
<xml_diff>
--- a/QA_TEST_MATRIX.xlsx
+++ b/QA_TEST_MATRIX.xlsx
@@ -560,7 +560,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Press and hold button (Panic Set)</t>
+          <t>Press the RED panic button</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -570,22 +570,26 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Immediate emergency trigger.</t>
+          <t>Tests IAS Zone panic activation mapping.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Release button (Panic Clear)</t>
+          <t>Press the RED panic button again</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ALL SIRENS STOP immediately.</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
+          <t>ALL SIRENS STOP.</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Tests IAS Zone panic clear mapping.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -595,7 +599,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Prints Battery/Voltage &amp; Temperature.</t>
+          <t>Prints Battery/Voltage.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">

</xml_diff>